<commit_message>
[MOSIP-32075]: Updated Templates for PMS
Signed-off-by: Chetan Kumar Hirematha <chetankumar.h.239@gmail.com>
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/template_type.xlsx
+++ b/mosip_master/xlsx/template_type.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\Mosip\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D493FBBA-311F-4FC6-980D-93205FF0EC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0689B7E-5B89-49DA-B78B-BBC2C72FF3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15468" uniqueCount="1497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15540" uniqueCount="1511">
   <si>
     <t>lang_code</t>
   </si>
@@ -6131,6 +6131,48 @@
   </si>
   <si>
     <t>எஸ்பிஐ காலாவதிக்கான பாட வார்ப்புரு</t>
+  </si>
+  <si>
+    <t>MISP_LICENSE_KEY_EXPIRY_TEMPLATE</t>
+  </si>
+  <si>
+    <t>Template for MISP License Key expiry</t>
+  </si>
+  <si>
+    <t>Modèle pour l'expiration de la clé de licence MISP</t>
+  </si>
+  <si>
+    <t>قالب لانتهاء صلاحية مفتاح ترخيص MISP</t>
+  </si>
+  <si>
+    <t>MISP लाइसेंस कुंजी समाप्ति के लिए टेम्पलेट</t>
+  </si>
+  <si>
+    <t>MISP ಲೈಸೆನ್ಸ್ ಕೀ ಅವಧಿ ಮುಗಿಯುವ ಟೆಂಪ್ಲೇಟ್</t>
+  </si>
+  <si>
+    <t>MISP உரிமக் கீ காலாவதிக்கான டெம்ப்ளேட்</t>
+  </si>
+  <si>
+    <t>MISP_LICENSE_KEY_EXPIRY_SUBJECT</t>
+  </si>
+  <si>
+    <t>Subject template for MISP License Key expiry</t>
+  </si>
+  <si>
+    <t>Modèle de sujet pour l'expiration de la clé de licence MISP</t>
+  </si>
+  <si>
+    <t>قالب موضوع لانتهاء صلاحية مفتاح ترخيص MISP</t>
+  </si>
+  <si>
+    <t>MISP ಲೈಸೆನ್ಸ್ ಕೀ ಅವಧಿ ಮುಗಿಯುವ ವಿಷಯ ಟೆಂಪ್ಲೇಟ್</t>
+  </si>
+  <si>
+    <t>MISP உரிமக் கீ காலாவதிக்கான பொருள் டெம்ப்ளேட்</t>
+  </si>
+  <si>
+    <t>MISP लाइसेंस कुंजी समाप्ति के लिए विषय टेम्पलेट</t>
   </si>
 </sst>
 </file>
@@ -6599,12 +6641,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2578"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:F2590"/>
+  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="10.140625" customWidth="1"/>
-    <col min="2" max="2" width="40.42578125" customWidth="1"/>
-    <col min="3" max="3" width="66.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" customWidth="1"/>
+    <col min="2" max="2" width="40.453125" customWidth="1"/>
+    <col min="3" max="3" width="66.7265625" customWidth="1"/>
     <col min="4" max="4" width="27" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12388,7 +12430,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="290" spans="1:6">
+    <row r="290" spans="1:6" ht="15">
       <c r="A290" s="5" t="s">
         <v>297</v>
       </c>
@@ -13148,7 +13190,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="328" spans="1:6" ht="30">
+    <row r="328" spans="1:6">
       <c r="A328" t="s">
         <v>297</v>
       </c>
@@ -15528,7 +15570,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="447" spans="1:6" ht="30">
+    <row r="447" spans="1:6">
       <c r="A447" t="s">
         <v>299</v>
       </c>
@@ -15628,7 +15670,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="452" spans="1:6" ht="30">
+    <row r="452" spans="1:6">
       <c r="A452" t="s">
         <v>299</v>
       </c>
@@ -15648,7 +15690,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="453" spans="1:6" ht="30">
+    <row r="453" spans="1:6">
       <c r="A453" t="s">
         <v>299</v>
       </c>
@@ -15688,7 +15730,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="455" spans="1:6" ht="30">
+    <row r="455" spans="1:6" ht="29">
       <c r="A455" t="s">
         <v>299</v>
       </c>
@@ -15708,7 +15750,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="456" spans="1:6" ht="30">
+    <row r="456" spans="1:6" ht="29">
       <c r="A456" t="s">
         <v>299</v>
       </c>
@@ -15748,7 +15790,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="458" spans="1:6" ht="30">
+    <row r="458" spans="1:6" ht="29">
       <c r="A458" t="s">
         <v>299</v>
       </c>
@@ -15768,7 +15810,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="459" spans="1:6" ht="30">
+    <row r="459" spans="1:6" ht="29">
       <c r="A459" t="s">
         <v>299</v>
       </c>
@@ -15908,7 +15950,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="466" spans="1:6" ht="30">
+    <row r="466" spans="1:6" ht="29">
       <c r="A466" t="s">
         <v>299</v>
       </c>
@@ -16008,7 +16050,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="471" spans="1:6" ht="30">
+    <row r="471" spans="1:6" ht="29">
       <c r="A471" t="s">
         <v>299</v>
       </c>
@@ -16408,7 +16450,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="491" spans="1:6" ht="30">
+    <row r="491" spans="1:6" ht="29">
       <c r="A491" t="s">
         <v>299</v>
       </c>
@@ -16468,7 +16510,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="494" spans="1:6" ht="30">
+    <row r="494" spans="1:6" ht="29">
       <c r="A494" t="s">
         <v>299</v>
       </c>
@@ -16488,7 +16530,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="495" spans="1:6" ht="30">
+    <row r="495" spans="1:6" ht="29">
       <c r="A495" t="s">
         <v>299</v>
       </c>
@@ -16508,7 +16550,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="496" spans="1:6" ht="30">
+    <row r="496" spans="1:6" ht="29">
       <c r="A496" t="s">
         <v>299</v>
       </c>
@@ -16528,7 +16570,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="497" spans="1:6" ht="30">
+    <row r="497" spans="1:6" ht="29">
       <c r="A497" t="s">
         <v>299</v>
       </c>
@@ -16548,7 +16590,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="498" spans="1:6" ht="30">
+    <row r="498" spans="1:6" ht="29">
       <c r="A498" t="s">
         <v>299</v>
       </c>
@@ -16568,7 +16610,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="499" spans="1:6" ht="30">
+    <row r="499" spans="1:6">
       <c r="A499" t="s">
         <v>299</v>
       </c>
@@ -16588,7 +16630,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="500" spans="1:6" ht="30">
+    <row r="500" spans="1:6">
       <c r="A500" t="s">
         <v>299</v>
       </c>
@@ -16608,7 +16650,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="501" spans="1:6" ht="30">
+    <row r="501" spans="1:6" ht="29">
       <c r="A501" t="s">
         <v>299</v>
       </c>
@@ -16628,7 +16670,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="502" spans="1:6" ht="30">
+    <row r="502" spans="1:6" ht="29">
       <c r="A502" t="s">
         <v>299</v>
       </c>
@@ -16668,7 +16710,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="504" spans="1:6" ht="30">
+    <row r="504" spans="1:6" ht="29">
       <c r="A504" t="s">
         <v>299</v>
       </c>
@@ -16688,7 +16730,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="505" spans="1:6" ht="30">
+    <row r="505" spans="1:6">
       <c r="A505" t="s">
         <v>299</v>
       </c>
@@ -16708,7 +16750,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="506" spans="1:6" ht="30">
+    <row r="506" spans="1:6" ht="29">
       <c r="A506" t="s">
         <v>299</v>
       </c>
@@ -16728,7 +16770,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="507" spans="1:6" ht="30">
+    <row r="507" spans="1:6" ht="29">
       <c r="A507" t="s">
         <v>299</v>
       </c>
@@ -16748,7 +16790,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="508" spans="1:6" ht="30">
+    <row r="508" spans="1:6" ht="29">
       <c r="A508" t="s">
         <v>299</v>
       </c>
@@ -16768,7 +16810,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="509" spans="1:6" ht="30">
+    <row r="509" spans="1:6" ht="29">
       <c r="A509" t="s">
         <v>299</v>
       </c>
@@ -58165,6 +58207,246 @@
         <v>1391</v>
       </c>
       <c r="F2578" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2579" spans="1:6">
+      <c r="A2579" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2579" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2579" t="s">
+        <v>1498</v>
+      </c>
+      <c r="D2579" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2579" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2579" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2580" spans="1:6">
+      <c r="A2580" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2580" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2580" t="s">
+        <v>1499</v>
+      </c>
+      <c r="D2580" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2580" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2580" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2581" spans="1:6">
+      <c r="A2581" t="s">
+        <v>291</v>
+      </c>
+      <c r="B2581" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2581" t="s">
+        <v>1500</v>
+      </c>
+      <c r="D2581" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2581" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2581" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2582" spans="1:6">
+      <c r="A2582" t="s">
+        <v>298</v>
+      </c>
+      <c r="B2582" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2582" t="s">
+        <v>1501</v>
+      </c>
+      <c r="D2582" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2582" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2582" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2583" spans="1:6">
+      <c r="A2583" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2583" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2583" t="s">
+        <v>1502</v>
+      </c>
+      <c r="D2583" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2583" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2583" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2584" spans="1:6">
+      <c r="A2584" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2584" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C2584" t="s">
+        <v>1503</v>
+      </c>
+      <c r="D2584" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2584" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2584" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2585" spans="1:6">
+      <c r="A2585" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2585" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2585" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D2585" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2585" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2585" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2586" spans="1:6">
+      <c r="A2586" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2586" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2586" t="s">
+        <v>1506</v>
+      </c>
+      <c r="D2586" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2586" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2586" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2587" spans="1:6">
+      <c r="A2587" t="s">
+        <v>291</v>
+      </c>
+      <c r="B2587" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2587" t="s">
+        <v>1507</v>
+      </c>
+      <c r="D2587" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2587" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2587" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2588" spans="1:6">
+      <c r="A2588" t="s">
+        <v>298</v>
+      </c>
+      <c r="B2588" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2588" t="s">
+        <v>1510</v>
+      </c>
+      <c r="D2588" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2588" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2588" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2589" spans="1:6">
+      <c r="A2589" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2589" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2589" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D2589" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2589" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2589" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="2590" spans="1:6">
+      <c r="A2590" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2590" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C2590" t="s">
+        <v>1509</v>
+      </c>
+      <c r="D2590" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2590" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F2590" t="s">
         <v>1392</v>
       </c>
     </row>

</xml_diff>